<commit_message>
OrderApproval.xlsx completo: Plantillas, Respuestas y Config
El libro incluye ahora todas las hojas de la propuesta sin desarrollo:
tblPlantillas con las tres plantillas, tblRespuestas con Folio, EnviarUTC,
Para, Asunto y Cuerpo como columnas calculadas y listas desplegables, y
Config (horas UTC y correo del operador). Instrucciones actualizada con los
flujos OA-A, OA-B y las reglas de Outlook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UfNaB1a2vwt4VqDwfvAyow
</commit_message>
<xml_diff>
--- a/docs/OrderApproval.xlsx
+++ b/docs/OrderApproval.xlsx
@@ -11,6 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MaterialOH" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buscar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plantillas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respuestas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="OH_Item">tblOH[Item]</definedName>
@@ -150,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -189,6 +192,18 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -335,6 +350,45 @@
     <tableColumn id="16" name="Etiqueta">
       <calculatedColumnFormula>"["&amp;tblCorreos[[#This Row],[Resultado]]&amp;"] BO# "&amp;IF(tblCorreos[[#This Row],[BO]]="","SIN BO#",tblCorreos[[#This Row],[BO]])&amp;IF(tblCorreos[[#This Row],[Prioridad]]="CRITICA"," · CRITICA","")&amp;" · "&amp;tblCorreos[[#This Row],[Asunto]]</calculatedColumnFormula>
     </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblPlantillas" displayName="tblPlantillas" ref="A1:B4" headerRowCount="1">
+  <autoFilter ref="A1:B4"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Nombre"/>
+    <tableColumn id="2" name="Cuerpo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblRespuestas" displayName="tblRespuestas" ref="A1:I2" headerRowCount="1">
+  <autoFilter ref="A1:I2"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Folio">
+      <calculatedColumnFormula>ROW()-ROW(tblRespuestas[[#Headers],[Folio]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" name="BO"/>
+    <tableColumn id="3" name="Plantilla"/>
+    <tableColumn id="4" name="EnviarEl"/>
+    <tableColumn id="5" name="EnviarUTC">
+      <calculatedColumnFormula>IF(tblRespuestas[[#This Row],[EnviarEl]]="","",tblRespuestas[[#This Row],[EnviarEl]]+Config!$B$2/24)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" name="Para">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(tblRespuestas[[#This Row],[BO]],tblCorreos[BO],tblCorreos[Remitente],"",0,-1)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" name="Asunto">
+      <calculatedColumnFormula>"RE: "&amp;_xlfn.XLOOKUP(tblRespuestas[[#This Row],[BO]],tblCorreos[BO],tblCorreos[Asunto],"",0,-1)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" name="Cuerpo">
+      <calculatedColumnFormula>_xlfn.LET(_xlpm.p,_xlfn.XLOOKUP(tblRespuestas[[#This Row],[Plantilla]],tblPlantillas[Nombre],tblPlantillas[Cuerpo],""),_xlpm.d,_xlfn.XLOOKUP(tblRespuestas[[#This Row],[BO]],tblCorreos[BO],tblCorreos[Detalle],"",0,-1),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlpm.p,CHAR(10),"&lt;br&gt;"),"{BO}",tblRespuestas[[#This Row],[BO]]),"{DETALLE}",_xlpm.d))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" name="Estado"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -629,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -648,7 +702,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>OrderApproval · libro de análisis</t>
+          <t>OrderApproval · libro completo</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -658,7 +712,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Compara los correos sencillos de #DC-MMex Order Approval contra el Material OH y registra el resultado. No responde ni marca correos.</t>
+          <t>Compara los correos de #DC-MMex Order Approval contra el Material OH, registra el resultado y prepara respuestas. Incluye todas las hojas de la propuesta sin desarrollo.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -754,187 +808,187 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="1" t="n"/>
-      <c r="C10" s="1" t="n"/>
-      <c r="D10" s="1" t="n"/>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Plantillas (tabla tblPlantillas)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Textos de respuesta: Aprobada, Shortage, En revisión. {BO} y {DETALLE} se reemplazan solos.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Editas los textos si quieres. Para un salto de línea dentro de la celda: Alt + Enter.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Nombres que usan las fórmulas (ya creados)</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="n"/>
-      <c r="D11" s="1" t="n"/>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Respuestas (tabla tblRespuestas)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Respuestas preparadas para enviar con el flujo OA-B. Para, Asunto y Cuerpo se arman solos a partir del BO# y la plantilla.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Escribes BO, Plantilla, EnviarEl (hora local) y Estado (amarillo). Cancelar = Estado «Cancelada».</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Apunta a</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Para qué</t>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>B2 = horas de diferencia con UTC (6 para Ciudad de México, Monterrey y Guadalajara). B3 = correo del operador.</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Ajustas B2 y B3 una vez.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>OH_Item</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>tblOH[Item]</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Número de artículo (no Item2).</t>
-        </is>
-      </c>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="n"/>
+      <c r="D13" s="1" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n"/>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>OH_Desc</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>tblOH[Item Description]</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Descripción que aparece en Detalle.</t>
-        </is>
-      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Nombres que usan las fórmulas (ya creados)</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="n"/>
+      <c r="D14" s="1" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>OH_Qty</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>tblOH[On-hand Qty]</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Existencia. Si un artículo está en varios Locator, se suma.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Apunta a</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Para qué</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Se ven en Fórmulas → Administrador de nombres. Si uno muestra #REF!, edítalo y en «Se refiere a» selecciona la columna con el mouse.</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="1" t="n"/>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>OH_Item</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>tblOH[Item]</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Número de artículo (no Item2).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
-      <c r="B17" s="1" t="n"/>
-      <c r="C17" s="1" t="n"/>
-      <c r="D17" s="1" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>OH_Desc</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>tblOH[Item Description]</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Descripción que aparece en Detalle.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Antes de usarlo</t>
-        </is>
-      </c>
-      <c r="C18" s="1" t="n"/>
-      <c r="D18" s="1" t="n"/>
-    </row>
-    <row r="19">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>OH_Qty</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>tblOH[On-hand Qty]</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Existencia. Si un artículo está en varios Locator, se suma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
       <c r="A19" s="1" t="n"/>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Paso</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Qué hacer</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Cómo saber que quedó</t>
-        </is>
-      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Se ven en Fórmulas → Administrador de nombres. Si uno muestra #REF!, edítalo y en «Se refiere a» selecciona la columna con el mouse.</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="n"/>
+      <c r="D19" s="1" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>1. Borrar ejemplos</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Hojas MaterialOH y Correos: selecciona las filas grises de ejemplo → clic derecho → Eliminar → Filas de la tabla.</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Las tablas quedan con el encabezado y una fila vacía.</t>
-        </is>
-      </c>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n"/>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>2. Pegar el Material OH</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Copia los datos del reporte desde la fila 2 (las 5 columnas, en el mismo orden) y pégalos en MaterialOH!A2 con Pegado especial → Valores.</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>En cualquier celda vacía, =SUM(OH_Qty) muestra la existencia total. Bórrala después.</t>
-        </is>
-      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Antes de usarlo</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="n"/>
+      <c r="D21" s="1" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>3. Conectar el flujo</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>En el flujo OA-A, acción «Agregar una fila a una tabla»: archivo OrderApproval.xlsx, tabla tblCorreos. Llena solo IdCorreo, Recibido, Remitente, Asunto, Cuerpo y Adjuntos.</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Al llegar un correo aparece un renglón nuevo y las columnas G–P se calculan solas.</t>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Paso</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Qué hacer</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Cómo saber que quedó</t>
         </is>
       </c>
     </row>
@@ -942,133 +996,311 @@
       <c r="A23" s="1" t="n"/>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>4. Cerrar Excel de escritorio</t>
+          <t>1. Borrar ejemplos</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Después de pegar el Material OH, guarda y cierra el libro.</t>
+          <t>Hojas MaterialOH y Correos: selecciona las filas grises de ejemplo → clic derecho → Eliminar → Filas de la tabla.</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Con el libro abierto, Power Automate puede marcarlo como bloqueado.</t>
+          <t>Las tablas quedan con el encabezado y una fila vacía.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="1" t="n"/>
-      <c r="C24" s="1" t="n"/>
-      <c r="D24" s="1" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>2. Pegar el Material OH</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Copia los datos del reporte desde la fila 2 (las 5 columnas, en el mismo orden) y pégalos en MaterialOH!A2 con Pegado especial → Valores.</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>En cualquier celda vacía, =SUM(OH_Qty) muestra la existencia total. Bórrala después.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Resultados</t>
-        </is>
-      </c>
-      <c r="C25" s="1" t="n"/>
-      <c r="D25" s="1" t="n"/>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>3. Conectar el flujo</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>En el flujo OA-A, acción «Agregar una fila a una tabla»: archivo OrderApproval.xlsx, tabla tblCorreos. Llena solo IdCorreo, Recibido, Remitente, Asunto, Cuerpo y Adjuntos.</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Al llegar un correo aparece un renglón nuevo y las columnas G–P se calculan solas.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Significado</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="n"/>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>4. Config</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Escribe en Config!B3 el correo del operador (ahí llegan los resúmenes del flujo OA-A).</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Config!B2 = 6 si estás en hora del centro de México.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n"/>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>VERDE</t>
+          <t>5. Respuestas</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Todos los artículos tienen existencia suficiente.</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="n"/>
+          <t>Borra la fila gris de ejemplo de Respuestas. Para programar una respuesta: nueva fila con BO, Plantilla, EnviarEl y Estado «Borrador», y ejecuta el flujo OA-B sobre esa fila.</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Para, Asunto y Cuerpo se llenan solos; el flujo cambia Estado a «Programada» y luego a «Enviada».</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>ROJO</t>
+          <t>6. Cerrar Excel de escritorio</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Falta material en al menos un artículo, o el asunto no trae BO#. Prioridad CRITICA si la RDD está a 7 días o menos.</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="n"/>
+          <t>Después de pegar el Material OH, guarda y cierra el libro.</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Con el libro abierto, Power Automate puede marcarlo como bloqueado.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n"/>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>NARANJA</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>Correo complejo (RE:/FW:, adjuntos, sin líneas Item / Qty) o formato no reconocido (Faltantes = -1). Revisión manual.</t>
-        </is>
-      </c>
+      <c r="B29" s="1" t="n"/>
+      <c r="C29" s="1" t="n"/>
       <c r="D29" s="1" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
-      <c r="B30" s="1" t="n"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Flujos de Power Automate que usan este libro</t>
+        </is>
+      </c>
       <c r="C30" s="1" t="n"/>
       <c r="D30" s="1" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Requisitos</t>
-        </is>
-      </c>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="n"/>
-    </row>
-    <row r="32" ht="28" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Flujo</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Qué hace</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Sección de la guía</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
       <c r="A32" s="1" t="n"/>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Excel de Microsoft 365 (escritorio o web). Las fórmulas usan LET, TEXTSPLIT, TEXTBEFORE, TEXTAFTER, XLOOKUP y FILTER, que no existen en Excel 2019 ni anteriores.</t>
-        </is>
-      </c>
-      <c r="C32" s="1" t="n"/>
-      <c r="D32" s="1" t="n"/>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>OA-A Clasificar correos</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Agrega cada correo a tblCorreos, lee Resultado, pone bandera en el buzón y envía al operador un resumen con Etiqueta y Detalle.</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Sección 5 (pasos 5.1 a 5.8)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n"/>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>OA-B Programar respuesta</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Envía a la hora EnviarUTC la respuesta de una fila de tblRespuestas si su Estado sigue en «Programada».</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Sección 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n"/>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Reglas de Outlook</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Colorean los resúmenes según [VERDE], [ROJO] o [NARANJA] en el asunto (columna Etiqueta).</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Sección 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n"/>
+      <c r="B35" s="1" t="n"/>
+      <c r="C35" s="1" t="n"/>
+      <c r="D35" s="1" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Resultados</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="n"/>
+      <c r="D36" s="1" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Significado</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n"/>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>VERDE</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Todos los artículos tienen existencia suficiente.</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n"/>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>ROJO</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Falta material en al menos un artículo, o el asunto no trae BO#. Prioridad CRITICA si la RDD está a 7 días o menos.</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n"/>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>NARANJA</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Correo complejo (RE:/FW:, adjuntos, sin líneas Item / Qty) o formato no reconocido (Faltantes = -1). Revisión manual.</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n"/>
+      <c r="B41" s="1" t="n"/>
+      <c r="C41" s="1" t="n"/>
+      <c r="D41" s="1" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n"/>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Requisitos</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="n"/>
+      <c r="D42" s="1" t="n"/>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="1" t="n"/>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Excel de Microsoft 365 (escritorio o web). Las fórmulas usan LET, TEXTSPLIT, TEXTBEFORE, TEXTAFTER, XLOOKUP y FILTER, que no existen en Excel 2019 ni anteriores. Los flujos usan los conectores estándar de Excel Online (Business) y Office 365 Outlook.</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="n"/>
+      <c r="D43" s="1" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n"/>
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>Guía completa: docs/PROPUESTA_SIN_DESARROLLO.md en el repositorio OA-JRM.</t>
         </is>
       </c>
-      <c r="C33" s="1" t="n"/>
-      <c r="D33" s="1" t="n"/>
+      <c r="C44" s="1" t="n"/>
+      <c r="D44" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B32:D32"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B43:D43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4667,10 +4899,302 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"Artículo,Contiene,Descripción"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Cuerpo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>{BO} y {DETALLE} se reemplazan solos. Salto de línea dentro de la celda: Alt + Enter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="135" customHeight="1">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>Hello,
+BO# {BO} has been reviewed. All requested items are available on hand and the order will be released.
+{DETALLE}
+Regards,
+Order Approval Team</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="135" customHeight="1">
+      <c r="A3" s="22" t="inlineStr">
+        <is>
+          <t>Shortage</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Hello,
+We reviewed BO# {BO}. Some items do not have enough on-hand inventory:
+{DETALLE}
+Please let us know if we should hold the order, ship partial, or substitute the items.
+Regards,
+Order Approval Team</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="135" customHeight="1">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Hello,
+We received your message about BO# {BO}. It is under review and we will follow up shortly.
+Regards,
+Order Approval Team</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Plantilla</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>EnviarEl</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>EnviarUTC</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Para</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Asunto</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Cuerpo</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>Amarillo/azul = escribes (BO, Plantilla, EnviarEl, Estado). Blanco = fórmula. Fila gris = ejemplo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="14">
+        <f>ROW()-ROW(tblRespuestas[[#Headers],[Folio]])</f>
+      </c>
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>93952630</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Shortage</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="n">
+        <v>46301.375</v>
+      </c>
+      <c r="E2" s="25">
+        <f>IF(tblRespuestas[[#This Row],[EnviarEl]]="","",tblRespuestas[[#This Row],[EnviarEl]]+Config!$B$2/24)</f>
+      </c>
+      <c r="F2" s="14">
+        <f>_xlfn.XLOOKUP(tblRespuestas[[#This Row],[BO]],tblCorreos[BO],tblCorreos[Remitente],"",0,-1)</f>
+      </c>
+      <c r="G2" s="14">
+        <f>"RE: "&amp;_xlfn.XLOOKUP(tblRespuestas[[#This Row],[BO]],tblCorreos[BO],tblCorreos[Asunto],"",0,-1)</f>
+      </c>
+      <c r="H2" s="14">
+        <f>_xlfn.LET(_xlpm.p,_xlfn.XLOOKUP(tblRespuestas[[#This Row],[Plantilla]],tblPlantillas[Nombre],tblPlantillas[Cuerpo],""),_xlpm.d,_xlfn.XLOOKUP(tblRespuestas[[#This Row],[BO]],tblCorreos[BO],tblCorreos[Detalle],"",0,-1),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlpm.p,CHAR(10),"&lt;br&gt;"),"{BO}",tblRespuestas[[#This Row],[BO]]),"{DETALLE}",_xlpm.d))</f>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>Programar: Estado «Borrador» → selecciona la fila → Automatizar → Power Automate → OA-B. Cancelar: Estado «Cancelada».</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
+      <formula1>INDIRECT("tblCorreos[BO]")</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
+      <formula1>INDIRECT("tblPlantillas[Nombre]")</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
+      <formula1>"Borrador,Programada,Enviada,Cancelada"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Parámetro</t>
+        </is>
+      </c>
+      <c r="B1" s="19" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Horas UTC</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Horas que se suman a la hora local para obtener UTC. Centro de México: 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Operador</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>operador@empresa.com</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Correo que recibe los resúmenes del flujo OA-A.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>